<commit_message>
data: atualiza posicao financeira 26-06-2026 — corrige cotacao USD
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Posição Financeira/Posição Financeira 26-06-2026.xlsx
+++ b/data/Posição Financeira/Posição Financeira 26-06-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailadventistas-my.sharepoint.com/personal/heber_elias_adventistas_org/Documents/pessoal/Projetos IA/VIGIA/data/Posição Financeira/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="203" documentId="8_{CA735DC7-0780-4D5B-902D-19CDAB62B616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D89E4E27-8186-420F-B1E2-C022276AC76F}"/>
+  <xr:revisionPtr revIDLastSave="205" documentId="8_{CA735DC7-0780-4D5B-902D-19CDAB62B616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD1BCC22-A942-4581-B9C1-C358B4537E77}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8AE765BB-1B3B-C94A-80E9-FD6B0D5051C9}"/>
   </bookViews>
@@ -781,7 +781,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="23"/>
                 <c:pt idx="0">
-                  <c:v>3184091713.8222747</c:v>
+                  <c:v>3187006399.3300352</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>3178670595.4822741</c:v>
@@ -822,31 +822,31 @@
                 <c:pt idx="13">
                   <c:v>3071929072.2587013</c:v>
                 </c:pt>
-                <c:pt idx="14" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="14" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>3066946423.4358106</c:v>
                 </c:pt>
-                <c:pt idx="15" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="15" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>3066172110.0887356</c:v>
                 </c:pt>
-                <c:pt idx="16" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="16" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>3017005263.7548132</c:v>
                 </c:pt>
-                <c:pt idx="17" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="17" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2978575355.9103217</c:v>
                 </c:pt>
-                <c:pt idx="18" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="18" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2957048188.1051764</c:v>
                 </c:pt>
-                <c:pt idx="19" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="19" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2939493750.6309209</c:v>
                 </c:pt>
-                <c:pt idx="20" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="20" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2892435615.0569272</c:v>
                 </c:pt>
-                <c:pt idx="21" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="21" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2884368597.8851318</c:v>
                 </c:pt>
-                <c:pt idx="22" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="22" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2858821590.3847275</c:v>
                 </c:pt>
               </c:numCache>
@@ -4635,23 +4635,23 @@
       </c>
       <c r="L17" s="16">
         <f>Somatória!C30</f>
-        <v>63474502.994399995</v>
+        <v>63719413.266199991</v>
       </c>
       <c r="M17" s="17">
         <f>Somatória!C30/Somatória!D30-1</f>
-        <v>3.3376649552565585E-3</v>
+        <v>7.2089469447043086E-3</v>
       </c>
       <c r="N17" s="17">
         <f>Somatória!C30/Somatória!G30-1</f>
-        <v>2.5550249233580846E-2</v>
+        <v>2.9507236345500454E-2</v>
       </c>
       <c r="O17" s="17">
         <f>Somatória!C30/Somatória!O30-1</f>
-        <v>-1.3846538841605693E-2</v>
+        <v>-1.0041560451619413E-2</v>
       </c>
       <c r="P17" s="17">
         <f>Somatória!C30/Somatória!Y30-1</f>
-        <v>-5.0540508900190906E-2</v>
+        <v>-4.6877110668481103E-2</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4687,23 +4687,23 @@
       </c>
       <c r="L18" s="16">
         <f>Somatória!C31</f>
-        <v>3120617210.8278747</v>
+        <v>3123286986.0638351</v>
       </c>
       <c r="M18" s="17">
         <f>Somatória!C31/Somatória!D31-1</f>
-        <v>1.6723227691777254E-3</v>
+        <v>2.5292814351098869E-3</v>
       </c>
       <c r="N18" s="17">
         <f>Somatória!C31/Somatória!G31-1</f>
-        <v>1.1983570463219406E-2</v>
+        <v>1.2849350689722927E-2</v>
       </c>
       <c r="O18" s="17">
         <f>Somatória!C31/Somatória!O31-1</f>
-        <v>3.8764703281317647E-2</v>
+        <v>3.9653395515401257E-2</v>
       </c>
       <c r="P18" s="17">
         <f>Somatória!C31/Somatória!Y31-1</f>
-        <v>0.11771226946555258</v>
+        <v>0.11866850354885972</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
@@ -4755,23 +4755,23 @@
       </c>
       <c r="L20" s="16">
         <f>SUM(L17:L19)</f>
-        <v>3184091713.8222747</v>
+        <v>3187006399.3300352</v>
       </c>
       <c r="M20" s="19">
         <f>Somatória!C32/Somatória!D32-1</f>
-        <v>1.7054671684777478E-3</v>
+        <v>2.6224182712133448E-3</v>
       </c>
       <c r="N20" s="19">
         <f>Somatória!C32/Somatória!G32-1</f>
-        <v>1.2250513344411296E-2</v>
+        <v>1.3177117276283123E-2</v>
       </c>
       <c r="O20" s="19">
         <f>Somatória!C32/Somatória!O32-1</f>
-        <v>3.7661124506918497E-2</v>
+        <v>3.861098905649718E-2</v>
       </c>
       <c r="P20" s="19">
         <f>Somatória!C32/Somatória!Y32-1</f>
-        <v>0.11377769236511681</v>
+        <v>0.11479723325481883</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -4788,7 +4788,7 @@
         <v>15</v>
       </c>
       <c r="L21" s="24">
-        <v>5.16</v>
+        <v>5.18</v>
       </c>
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
@@ -6203,7 +6203,7 @@
       <c r="B30" s="28"/>
       <c r="C30" s="28">
         <f t="shared" ref="C30:D30" si="78">C3+(C12*C35)+C21</f>
-        <v>63474502.994399995</v>
+        <v>63719413.266199991</v>
       </c>
       <c r="D30" s="28">
         <f t="shared" si="78"/>
@@ -6298,7 +6298,7 @@
       <c r="B31" s="28"/>
       <c r="C31" s="28">
         <f t="shared" ref="C31:D31" si="90">C4+(C13*C35)+C22</f>
-        <v>3120617210.8278747</v>
+        <v>3123286986.0638351</v>
       </c>
       <c r="D31" s="28">
         <f t="shared" si="90"/>
@@ -6392,7 +6392,7 @@
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="C32">
         <f t="shared" ref="C32" si="103">SUM(C30:C31)</f>
-        <v>3184091713.8222747</v>
+        <v>3187006399.3300352</v>
       </c>
       <c r="D32">
         <f t="shared" ref="D32:E32" si="104">SUM(D30:D31)</f>
@@ -6491,7 +6491,7 @@
         <v>26</v>
       </c>
       <c r="C35">
-        <v>5.16</v>
+        <v>5.18</v>
       </c>
       <c r="D35">
         <v>5.16</v>
@@ -9284,14 +9284,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="546f6921-c430-45e7-8b30-d6d9b86d8f0f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="364167a4-bc77-49ec-93f2-879d4481bae7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9550,21 +9548,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="546f6921-c430-45e7-8b30-d6d9b86d8f0f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="364167a4-bc77-49ec-93f2-879d4481bae7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95E1F151-0F5C-495E-9947-EE9B49CBAA94}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5656E7FC-8739-4AA4-8E2F-8E1DDD7713FD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="546f6921-c430-45e7-8b30-d6d9b86d8f0f"/>
-    <ds:schemaRef ds:uri="364167a4-bc77-49ec-93f2-879d4481bae7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9589,9 +9586,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5656E7FC-8739-4AA4-8E2F-8E1DDD7713FD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95E1F151-0F5C-495E-9947-EE9B49CBAA94}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="546f6921-c430-45e7-8b30-d6d9b86d8f0f"/>
+    <ds:schemaRef ds:uri="364167a4-bc77-49ec-93f2-879d4481bae7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>